<commit_message>
Change author_overlap_pct to measure replication team independence
Calculate as overlap/replication_authors instead of overlap/original_authors.
This better reflects how independent the replication team is:
- 0% = fully independent (no original authors on replication)
- 100% = not independent (all replication authors were on original)

Updated codebook description accordingly.

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipelines/fred/fred_codebook.xlsx
+++ b/pipelines/fred/fred_codebook.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -35,7 +35,7 @@
     <t xml:space="preserve">fred_id</t>
   </si>
   <si>
-    <t xml:space="preserve">Corresponding entry in the FORRT Replication Database (FReD), can be used to filter the crowdsourced FReD data for additional studies.</t>
+    <t xml:space="preserve">Corresponding entry in the FORRT Replication Database (FReD) 1.0, can be used to filter the crowdsourced FReD data for additional entries (though this is not generally recommended)</t>
   </si>
   <si>
     <t xml:space="preserve">ref_o</t>
@@ -86,7 +86,7 @@
     <t xml:space="preserve">author_overlap_pct</t>
   </si>
   <si>
-    <t xml:space="preserve">Percentage of original study authors who are also replication authors (based on family name matching). NA if author data unavailable for either study.</t>
+    <t xml:space="preserve">Percentage of replication study authors who are also original study authors (measures independence of replication team; 0% = fully independent)</t>
   </si>
   <si>
     <t xml:space="preserve">discipline</t>
@@ -128,7 +128,7 @@
     <t xml:space="preserve">es_value_o</t>
   </si>
   <si>
-    <t xml:space="preserve">original effect size value, contains values unless it is a test statistic (then contains entire report, e.g. in the form of F(df1, df2) = value)</t>
+    <t xml:space="preserve">original effect size value, contains numers only unless it is a test statistic (then contains entire report, e.g. in the form of F(df1, df2) = value)</t>
   </si>
   <si>
     <t xml:space="preserve">es_type_o</t>
@@ -170,7 +170,7 @@
     <t xml:space="preserve">prereg_o</t>
   </si>
   <si>
-    <t xml:space="preserve">Link to preregistration of O</t>
+    <t xml:space="preserve">Link to preregistration of original</t>
   </si>
   <si>
     <t xml:space="preserve">n_r</t>
@@ -182,7 +182,7 @@
     <t xml:space="preserve">es_value_r</t>
   </si>
   <si>
-    <t xml:space="preserve">replication effect size value, contains values unless it is a test statistic (then contains entire report, e.g. in the form of F(df1, df2) = value)</t>
+    <t xml:space="preserve">replication effect size value, contains numbers only unless it is a test statistic (then contains entire report, e.g. in the form of F(df1, df2) = value)</t>
   </si>
   <si>
     <t xml:space="preserve">es_type_r</t>
@@ -206,9 +206,6 @@
     <t xml:space="preserve">pval_type_r</t>
   </si>
   <si>
-    <t xml:space="preserve">How is p-val reported? "=" (e) / "&lt;" (l) / "&gt;" (g) or combined (le, ge)? for example "p &lt;= .05" should be coded as "le"</t>
-  </si>
-  <si>
     <t xml:space="preserve">pval_tails_r</t>
   </si>
   <si>
@@ -225,7 +222,7 @@
   </si>
   <si>
     <t xml:space="preserve">Outcome based on the narrative interpretation of the replication authors (successful, failed, mixed, uninformative, 
-statistically successful but flawed)</t>
+statistically successful but flawed, descriptive only)</t>
   </si>
   <si>
     <t xml:space="preserve">reported_success_quote</t>
@@ -935,12 +932,12 @@
         <v>63</v>
       </c>
       <c r="B33" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
         <v>48</v>
@@ -948,7 +945,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B35" t="s">
         <v>50</v>
@@ -956,178 +953,178 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
+        <v>66</v>
+      </c>
+      <c r="B36" t="s">
         <v>67</v>
-      </c>
-      <c r="B36" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" t="s">
         <v>69</v>
-      </c>
-      <c r="B37" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38" t="s">
         <v>71</v>
-      </c>
-      <c r="B38" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" t="s">
         <v>73</v>
-      </c>
-      <c r="B39" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
+        <v>74</v>
+      </c>
+      <c r="B40" t="s">
         <v>75</v>
-      </c>
-      <c r="B40" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
+        <v>76</v>
+      </c>
+      <c r="B41" t="s">
         <v>77</v>
-      </c>
-      <c r="B41" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
         <v>79</v>
-      </c>
-      <c r="B42" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
+        <v>80</v>
+      </c>
+      <c r="B43" t="s">
         <v>81</v>
-      </c>
-      <c r="B43" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
+        <v>82</v>
+      </c>
+      <c r="B44" t="s">
         <v>83</v>
-      </c>
-      <c r="B44" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
+        <v>84</v>
+      </c>
+      <c r="B45" t="s">
         <v>85</v>
-      </c>
-      <c r="B45" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
+        <v>86</v>
+      </c>
+      <c r="B46" t="s">
         <v>87</v>
-      </c>
-      <c r="B46" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
+        <v>88</v>
+      </c>
+      <c r="B47" t="s">
         <v>89</v>
-      </c>
-      <c r="B47" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
+        <v>90</v>
+      </c>
+      <c r="B48" t="s">
         <v>91</v>
-      </c>
-      <c r="B48" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
+        <v>92</v>
+      </c>
+      <c r="B49" t="s">
         <v>93</v>
-      </c>
-      <c r="B49" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
+        <v>94</v>
+      </c>
+      <c r="B50" t="s">
         <v>95</v>
-      </c>
-      <c r="B50" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
+        <v>96</v>
+      </c>
+      <c r="B51" t="s">
         <v>97</v>
-      </c>
-      <c r="B51" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
+        <v>98</v>
+      </c>
+      <c r="B52" t="s">
         <v>99</v>
-      </c>
-      <c r="B52" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
+        <v>100</v>
+      </c>
+      <c r="B53" t="s">
         <v>101</v>
-      </c>
-      <c r="B53" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
+        <v>102</v>
+      </c>
+      <c r="B54" t="s">
         <v>103</v>
-      </c>
-      <c r="B54" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
+        <v>104</v>
+      </c>
+      <c r="B55" t="s">
         <v>105</v>
-      </c>
-      <c r="B55" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
+        <v>106</v>
+      </c>
+      <c r="B56" t="s">
         <v>107</v>
-      </c>
-      <c r="B56" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
+        <v>108</v>
+      </c>
+      <c r="B57" t="s">
         <v>109</v>
-      </c>
-      <c r="B57" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>